<commit_message>
Refresh sample workbook with recovered 7/27 origination scores
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-27_new.xlsx
+++ b/reports/universe_2026-07-27_new.xlsx
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28 11:26 local</t>
+          <t>2026-07-28 12:36 local</t>
         </is>
       </c>
     </row>
@@ -25225,7 +25225,7 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>2026-07-28 11:26 local</t>
+          <t>2026-07-28 12:36 local</t>
         </is>
       </c>
     </row>
@@ -27778,8 +27778,14 @@
       <c r="P3" s="19" t="n"/>
       <c r="Q3" s="19" t="n"/>
       <c r="R3" s="19" t="n"/>
-      <c r="S3" s="19" t="n"/>
-      <c r="T3" s="19" t="n"/>
+      <c r="S3" s="21" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="T3" s="19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U3" s="19" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -27849,8 +27855,14 @@
       <c r="P4" s="19" t="n"/>
       <c r="Q4" s="19" t="n"/>
       <c r="R4" s="19" t="n"/>
-      <c r="S4" s="19" t="n"/>
-      <c r="T4" s="19" t="n"/>
+      <c r="S4" s="21" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="T4" s="19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U4" s="19" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -27991,8 +28003,14 @@
       <c r="P6" s="19" t="n"/>
       <c r="Q6" s="19" t="n"/>
       <c r="R6" s="19" t="n"/>
-      <c r="S6" s="19" t="n"/>
-      <c r="T6" s="19" t="n"/>
+      <c r="S6" s="21" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="T6" s="19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U6" s="19" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -28062,8 +28080,14 @@
       <c r="P7" s="19" t="n"/>
       <c r="Q7" s="19" t="n"/>
       <c r="R7" s="19" t="n"/>
-      <c r="S7" s="19" t="n"/>
-      <c r="T7" s="19" t="n"/>
+      <c r="S7" s="21" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="T7" s="19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U7" s="19" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -28133,8 +28157,14 @@
       <c r="P8" s="19" t="n"/>
       <c r="Q8" s="19" t="n"/>
       <c r="R8" s="19" t="n"/>
-      <c r="S8" s="19" t="n"/>
-      <c r="T8" s="19" t="n"/>
+      <c r="S8" s="21" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="T8" s="19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U8" s="19" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -28275,8 +28305,14 @@
       <c r="P10" s="19" t="n"/>
       <c r="Q10" s="19" t="n"/>
       <c r="R10" s="19" t="n"/>
-      <c r="S10" s="19" t="n"/>
-      <c r="T10" s="19" t="n"/>
+      <c r="S10" s="21" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="T10" s="19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="U10" s="19" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -28346,8 +28382,14 @@
       <c r="P11" s="19" t="n"/>
       <c r="Q11" s="19" t="n"/>
       <c r="R11" s="19" t="n"/>
-      <c r="S11" s="19" t="n"/>
-      <c r="T11" s="19" t="n"/>
+      <c r="S11" s="21" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="T11" s="19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U11" s="19" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -28425,8 +28467,14 @@
       <c r="P12" s="19" t="n"/>
       <c r="Q12" s="19" t="n"/>
       <c r="R12" s="19" t="n"/>
-      <c r="S12" s="19" t="n"/>
-      <c r="T12" s="19" t="n"/>
+      <c r="S12" s="21" t="n">
+        <v>49</v>
+      </c>
+      <c r="T12" s="19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="U12" s="19" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -28575,8 +28623,14 @@
       <c r="P14" s="24" t="n"/>
       <c r="Q14" s="24" t="n"/>
       <c r="R14" s="24" t="n"/>
-      <c r="S14" s="24" t="n"/>
-      <c r="T14" s="24" t="n"/>
+      <c r="S14" s="26" t="n">
+        <v>59</v>
+      </c>
+      <c r="T14" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U14" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -28646,8 +28700,14 @@
       <c r="P15" s="24" t="n"/>
       <c r="Q15" s="24" t="n"/>
       <c r="R15" s="24" t="n"/>
-      <c r="S15" s="24" t="n"/>
-      <c r="T15" s="24" t="n"/>
+      <c r="S15" s="26" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="T15" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U15" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -28717,8 +28777,14 @@
       <c r="P16" s="24" t="n"/>
       <c r="Q16" s="24" t="n"/>
       <c r="R16" s="24" t="n"/>
-      <c r="S16" s="24" t="n"/>
-      <c r="T16" s="24" t="n"/>
+      <c r="S16" s="26" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="T16" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U16" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -29151,8 +29217,14 @@
       <c r="P22" s="24" t="n"/>
       <c r="Q22" s="24" t="n"/>
       <c r="R22" s="24" t="n"/>
-      <c r="S22" s="24" t="n"/>
-      <c r="T22" s="24" t="n"/>
+      <c r="S22" s="26" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="T22" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U22" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -29222,8 +29294,14 @@
       <c r="P23" s="24" t="n"/>
       <c r="Q23" s="24" t="n"/>
       <c r="R23" s="24" t="n"/>
-      <c r="S23" s="24" t="n"/>
-      <c r="T23" s="24" t="n"/>
+      <c r="S23" s="26" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="T23" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U23" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -29293,8 +29371,14 @@
       <c r="P24" s="24" t="n"/>
       <c r="Q24" s="24" t="n"/>
       <c r="R24" s="24" t="n"/>
-      <c r="S24" s="24" t="n"/>
-      <c r="T24" s="24" t="n"/>
+      <c r="S24" s="26" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="T24" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U24" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -29364,8 +29448,14 @@
       <c r="P25" s="24" t="n"/>
       <c r="Q25" s="24" t="n"/>
       <c r="R25" s="24" t="n"/>
-      <c r="S25" s="24" t="n"/>
-      <c r="T25" s="24" t="n"/>
+      <c r="S25" s="26" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="T25" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U25" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -29435,8 +29525,14 @@
       <c r="P26" s="24" t="n"/>
       <c r="Q26" s="24" t="n"/>
       <c r="R26" s="24" t="n"/>
-      <c r="S26" s="24" t="n"/>
-      <c r="T26" s="24" t="n"/>
+      <c r="S26" s="26" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="T26" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U26" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -29514,8 +29610,14 @@
       <c r="P27" s="24" t="n"/>
       <c r="Q27" s="24" t="n"/>
       <c r="R27" s="24" t="n"/>
-      <c r="S27" s="24" t="n"/>
-      <c r="T27" s="24" t="n"/>
+      <c r="S27" s="26" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="T27" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U27" s="24" t="inlineStr">
         <is>
           <t>REPAIR</t>
@@ -29656,8 +29758,14 @@
       <c r="P29" s="24" t="n"/>
       <c r="Q29" s="24" t="n"/>
       <c r="R29" s="24" t="n"/>
-      <c r="S29" s="24" t="n"/>
-      <c r="T29" s="24" t="n"/>
+      <c r="S29" s="26" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="T29" s="24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="U29" s="24" t="inlineStr">
         <is>
           <t>REPAIR</t>
@@ -29727,8 +29835,14 @@
       <c r="P30" s="24" t="n"/>
       <c r="Q30" s="24" t="n"/>
       <c r="R30" s="24" t="n"/>
-      <c r="S30" s="24" t="n"/>
-      <c r="T30" s="24" t="n"/>
+      <c r="S30" s="26" t="n">
+        <v>49</v>
+      </c>
+      <c r="T30" s="24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="U30" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -29798,8 +29912,14 @@
       <c r="P31" s="24" t="n"/>
       <c r="Q31" s="24" t="n"/>
       <c r="R31" s="24" t="n"/>
-      <c r="S31" s="24" t="n"/>
-      <c r="T31" s="24" t="n"/>
+      <c r="S31" s="26" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="T31" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U31" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -30098,8 +30218,14 @@
       <c r="P35" s="24" t="n"/>
       <c r="Q35" s="24" t="n"/>
       <c r="R35" s="24" t="n"/>
-      <c r="S35" s="24" t="n"/>
-      <c r="T35" s="24" t="n"/>
+      <c r="S35" s="26" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="T35" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U35" s="24" t="inlineStr">
         <is>
           <t>REPAIR</t>
@@ -30240,8 +30366,14 @@
       <c r="P37" s="24" t="n"/>
       <c r="Q37" s="24" t="n"/>
       <c r="R37" s="24" t="n"/>
-      <c r="S37" s="24" t="n"/>
-      <c r="T37" s="24" t="n"/>
+      <c r="S37" s="26" t="n">
+        <v>65</v>
+      </c>
+      <c r="T37" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U37" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -30311,8 +30443,14 @@
       <c r="P38" s="24" t="n"/>
       <c r="Q38" s="24" t="n"/>
       <c r="R38" s="24" t="n"/>
-      <c r="S38" s="24" t="n"/>
-      <c r="T38" s="24" t="n"/>
+      <c r="S38" s="26" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="T38" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U38" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -30524,8 +30662,14 @@
       <c r="P41" s="24" t="n"/>
       <c r="Q41" s="24" t="n"/>
       <c r="R41" s="24" t="n"/>
-      <c r="S41" s="24" t="n"/>
-      <c r="T41" s="24" t="n"/>
+      <c r="S41" s="26" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="T41" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U41" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -30666,8 +30810,14 @@
       <c r="P43" s="24" t="n"/>
       <c r="Q43" s="24" t="n"/>
       <c r="R43" s="24" t="n"/>
-      <c r="S43" s="24" t="n"/>
-      <c r="T43" s="24" t="n"/>
+      <c r="S43" s="26" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="T43" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U43" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -30745,8 +30895,14 @@
       <c r="P44" s="24" t="n"/>
       <c r="Q44" s="24" t="n"/>
       <c r="R44" s="24" t="n"/>
-      <c r="S44" s="24" t="n"/>
-      <c r="T44" s="24" t="n"/>
+      <c r="S44" s="26" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="T44" s="24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="U44" s="24" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -30887,8 +31043,14 @@
       <c r="P46" s="24" t="n"/>
       <c r="Q46" s="24" t="n"/>
       <c r="R46" s="24" t="n"/>
-      <c r="S46" s="24" t="n"/>
-      <c r="T46" s="24" t="n"/>
+      <c r="S46" s="26" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="T46" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="U46" s="24" t="inlineStr">
         <is>
           <t>PASS</t>

</xml_diff>